<commit_message>
Sync order template figures
</commit_message>
<xml_diff>
--- a/周维度经营看板上传模板.xlsx
+++ b/周维度经营看板上传模板.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="21000" windowHeight="14005" firstSheet="1" activeTab="7"/>
+    <workbookView windowWidth="21000" windowHeight="11074"/>
   </bookViews>
   <sheets>
     <sheet name="订单数据" sheetId="1" r:id="rId1"/>
@@ -82,7 +82,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="81">
   <si>
     <t>周次</t>
   </si>
@@ -328,6 +328,12 @@
   </si>
   <si>
     <t>KEY-SKY断货率进一步降低到2%，新下单金额上涨81%，7月廊坊仓面积从1300平降低到1100平</t>
+  </si>
+  <si>
+    <t>08-01</t>
+  </si>
+  <si>
+    <t>08-10</t>
   </si>
 </sst>
 </file>
@@ -1035,7 +1041,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1121,6 +1127,22 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment/>
+      <extLst>
+        <ext xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" uri="{F19249F5-4A6E-446B-B59F-E2C9F2DAA1D5}">
+          <etc:displayText val="2"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment/>
+      <extLst>
+        <ext xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" uri="{F19249F5-4A6E-446B-B59F-E2C9F2DAA1D5}">
+          <etc:displayText val="2"/>
+        </ext>
+      </extLst>
     </xf>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1" quotePrefix="1"/>
@@ -1522,17 +1544,17 @@
       <c r="A3" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="1">
+      <c r="B3" s="36">
         <v>4684</v>
       </c>
-      <c r="C3" s="23">
-        <v>11875244.04</v>
-      </c>
-      <c r="D3" s="1">
-        <v>1981</v>
-      </c>
-      <c r="E3" s="23">
-        <v>15540809.43</v>
+      <c r="C3" s="37">
+        <v>8243621.3</v>
+      </c>
+      <c r="D3" s="36">
+        <v>1917</v>
+      </c>
+      <c r="E3" s="37">
+        <v>11528192.33</v>
       </c>
       <c r="F3" s="1">
         <v>98</v>
@@ -1546,9 +1568,9 @@
       <c r="I3" s="1">
         <v>3925227.65</v>
       </c>
-      <c r="J3" s="36">
+      <c r="J3" s="38">
         <f>(C3-C2)/C2</f>
-        <v>0.807144085584268</v>
+        <v>0.254493080387382</v>
       </c>
     </row>
   </sheetData>
@@ -1677,7 +1699,7 @@
       </c>
     </row>
     <row r="4" customHeight="1" spans="1:11">
-      <c r="A4" s="37" t="s">
+      <c r="A4" s="39" t="s">
         <v>23</v>
       </c>
       <c r="B4" s="29">
@@ -1785,7 +1807,7 @@
       </c>
     </row>
     <row r="4" customHeight="1" spans="1:5">
-      <c r="A4" s="38" t="s">
+      <c r="A4" s="40" t="s">
         <v>23</v>
       </c>
       <c r="B4" s="5">
@@ -1859,7 +1881,7 @@
       </c>
     </row>
     <row r="4" customHeight="1" spans="1:4">
-      <c r="A4" s="38" t="s">
+      <c r="A4" s="40" t="s">
         <v>23</v>
       </c>
       <c r="B4" s="7">
@@ -2001,7 +2023,7 @@
       </c>
     </row>
     <row r="3" customHeight="1" spans="1:17">
-      <c r="A3" s="39" t="s">
+      <c r="A3" s="41" t="s">
         <v>51</v>
       </c>
       <c r="B3" s="19">
@@ -2446,8 +2468,8 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" customHeight="1" outlineLevelRow="1" outlineLevelCol="1"/>
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" customHeight="1" outlineLevelRow="3" outlineLevelCol="1"/>
   <cols>
     <col min="2" max="2" width="28.5038759689922" style="1" customWidth="1"/>
     <col min="3" max="3" width="19.1627906976744" style="1" customWidth="1"/>
@@ -2470,6 +2492,22 @@
         <v>78</v>
       </c>
     </row>
+    <row r="3" customHeight="1" spans="1:2">
+      <c r="A3" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B3" s="1">
+        <v>2222</v>
+      </c>
+    </row>
+    <row r="4" customHeight="1" spans="1:2">
+      <c r="A4" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B4" s="1">
+        <v>666</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>

</xml_diff>